<commit_message>
Bulls launch sheet: add Ulys domain and digidip link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhuR34CyHmHAyLdYHXxuU5
</commit_message>
<xml_diff>
--- a/media_buyer/Bulls_3_offers_2026-10-11.xlsx
+++ b/media_buyer/Bulls_3_offers_2026-10-11.xlsx
@@ -473,14 +473,14 @@
           <t>FR</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ulys.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fulys.com&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Bulls launch sheet: add Virgin Voyages Impact link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhuR34CyHmHAyLdYHXxuU5
</commit_message>
<xml_diff>
--- a/media_buyer/Bulls_3_offers_2026-10-11.xlsx
+++ b/media_buyer/Bulls_3_offers_2026-10-11.xlsx
@@ -552,9 +552,9 @@
           <t>virginvoyages.com</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://virginvoyages.sjv.io/m4B0oe</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Bulls launch sheet: planned Elite Reads article URLs for the 3 offers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NhuR34CyHmHAyLdYHXxuU5
</commit_message>
<xml_diff>
--- a/media_buyer/Bulls_3_offers_2026-10-11.xlsx
+++ b/media_buyer/Bulls_3_offers_2026-10-11.xlsx
@@ -483,9 +483,9 @@
           <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fulys.com&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/ulys-toll-badge-france-guide/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -520,9 +520,9 @@
           <t>https://3425.digidip.net/visit?url=https%3A%2F%2Fwww.1und1.de&amp;currurl=https%3A%2F%2Felite-reads.com&amp;ref={clickid}</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/1und1-internet-mobile-tariffs/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -557,9 +557,9 @@
           <t>https://virginvoyages.sjv.io/m4B0oe</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>TO CONFIRM</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://www.elite-reads.com/virgin-voyages-adult-only-cruises-guide/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -567,7 +567,7 @@
           <t>Impact</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>NYJL - Impact - RDV - NY</t>
         </is>

</xml_diff>